<commit_message>
AI book: split AI into pack file 09_ai, add decision-flow/targets/constants
PACK["09_ai"] takes the 06_ai domain out of 04_che_do_kinh_te_ai (file list
19 -> 21, all pack checks and the sheet/md regrouping are PACK-derived so no
hand-kept list needed elsewhere); adds 6 new sheets built from a static read
of the AI code: decision flow per layer, tower/boss target scoring, AiSkill
per difficulty, anti-stuck constants, the aircraft rearm cycle, and every
named AI constant still inline in C#. export.py check --game-json: 21/21 PASS.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/export/current/08_tham_chieu.xlsx
+++ b/Docs/export/current/08_tham_chieu.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -621,7 +621,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
@@ -677,7 +677,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
@@ -733,7 +733,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -744,7 +744,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -789,7 +789,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -845,7 +845,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -957,7 +957,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="N21" t="inlineStr"/>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N24" t="inlineStr"/>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N32" t="inlineStr"/>
@@ -2293,7 +2293,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N36" t="inlineStr"/>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -2584,7 +2584,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N38" t="inlineStr"/>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N39" t="inlineStr"/>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N40" t="inlineStr"/>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N41" t="inlineStr"/>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N42" t="inlineStr"/>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N43" t="inlineStr"/>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N44" t="inlineStr"/>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N45" t="inlineStr"/>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N46" t="inlineStr"/>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N47" t="inlineStr"/>
@@ -3153,7 +3153,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N48" t="inlineStr"/>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N50" t="inlineStr"/>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu;04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu;09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu; 09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N52" t="inlineStr"/>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N54" t="inlineStr"/>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N55" t="inlineStr"/>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N56" t="inlineStr"/>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N57" t="inlineStr"/>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N58" t="inlineStr"/>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K59" t="inlineStr"/>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N59" t="inlineStr"/>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N62" t="inlineStr"/>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu;04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu;09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu; 09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N63" t="inlineStr"/>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N64" t="inlineStr"/>
@@ -4109,7 +4109,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N65" t="inlineStr"/>
@@ -4165,7 +4165,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K66" t="inlineStr"/>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N66" t="inlineStr"/>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N67" t="inlineStr"/>
@@ -4273,7 +4273,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N68" t="inlineStr"/>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N69" t="inlineStr"/>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N70" t="inlineStr"/>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="N71" t="inlineStr"/>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N72" t="inlineStr"/>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N73" t="inlineStr"/>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N75" t="inlineStr"/>
@@ -4725,7 +4725,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N76" t="inlineStr"/>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N77" t="inlineStr"/>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N78" t="inlineStr"/>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -4912,7 +4912,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="N79" t="inlineStr"/>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="N80" t="inlineStr"/>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="N81" t="inlineStr"/>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="K82" t="inlineStr"/>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="N82" t="inlineStr"/>
@@ -15252,7 +15252,7 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="49" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -15319,7 +15319,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Arty</t>
+          <t>09_ai/AI_vai_tro/Arty</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -15334,7 +15334,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Arty)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Arty)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -15357,7 +15357,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/AttackHeli</t>
+          <t>09_ai/AI_vai_tro/AttackHeli</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -15372,7 +15372,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/AttackHeli)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/AttackHeli)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -15395,7 +15395,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Bomber</t>
+          <t>09_ai/AI_vai_tro/Bomber</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -15410,7 +15410,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Bomber)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Bomber)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -15433,7 +15433,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Bunker</t>
+          <t>09_ai/AI_vai_tro/Bunker</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -15448,7 +15448,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Bunker)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Bunker)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -15471,7 +15471,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/CAS</t>
+          <t>09_ai/AI_vai_tro/CAS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -15486,7 +15486,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/CAS)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/CAS)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -15509,7 +15509,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Drone</t>
+          <t>09_ai/AI_vai_tro/Drone</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -15524,7 +15524,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Drone)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Drone)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -15547,7 +15547,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Fighter</t>
+          <t>09_ai/AI_vai_tro/Fighter</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -15562,7 +15562,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Fighter)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Fighter)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -15585,7 +15585,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Flame</t>
+          <t>09_ai/AI_vai_tro/Flame</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -15600,7 +15600,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Flame)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Flame)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -15623,7 +15623,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Gunship</t>
+          <t>09_ai/AI_vai_tro/Gunship</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -15638,7 +15638,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Gunship)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Gunship)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -15661,7 +15661,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/GunshipHeli</t>
+          <t>09_ai/AI_vai_tro/GunshipHeli</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -15676,7 +15676,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/GunshipHeli)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/GunshipHeli)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -15699,7 +15699,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Heavy</t>
+          <t>09_ai/AI_vai_tro/Heavy</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -15714,7 +15714,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Heavy)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Heavy)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -15737,7 +15737,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/IFV</t>
+          <t>09_ai/AI_vai_tro/IFV</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -15752,7 +15752,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/IFV)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/IFV)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -15775,7 +15775,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Laser</t>
+          <t>09_ai/AI_vai_tro/Laser</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -15790,7 +15790,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Laser)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Laser)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -15813,7 +15813,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Light</t>
+          <t>09_ai/AI_vai_tro/Light</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -15828,7 +15828,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Light)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Light)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -15851,7 +15851,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/MBT</t>
+          <t>09_ai/AI_vai_tro/MBT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/MBT)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/MBT)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -15889,7 +15889,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/MLRS</t>
+          <t>09_ai/AI_vai_tro/MLRS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/MLRS)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/MLRS)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -15927,7 +15927,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Rail</t>
+          <t>09_ai/AI_vai_tro/Rail</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Rail)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Rail)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -15965,7 +15965,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Recon</t>
+          <t>09_ai/AI_vai_tro/Recon</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -15980,7 +15980,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Recon)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Recon)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -16003,7 +16003,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/SAM</t>
+          <t>09_ai/AI_vai_tro/SAM</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -16018,7 +16018,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/SAM)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/SAM)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -16041,7 +16041,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/ScoutHeli</t>
+          <t>09_ai/AI_vai_tro/ScoutHeli</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/ScoutHeli)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/ScoutHeli)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -16079,7 +16079,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Siege</t>
+          <t>09_ai/AI_vai_tro/Siege</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -16094,7 +16094,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Siege)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Siege)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -16117,7 +16117,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/SPAAG</t>
+          <t>09_ai/AI_vai_tro/SPAAG</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -16132,7 +16132,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/SPAAG)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/SPAAG)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -16155,7 +16155,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Stealth</t>
+          <t>09_ai/AI_vai_tro/Stealth</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -16170,7 +16170,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Stealth)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Stealth)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -16193,7 +16193,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Strike</t>
+          <t>09_ai/AI_vai_tro/Strike</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Strike)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Strike)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -16231,7 +16231,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/Support</t>
+          <t>09_ai/AI_vai_tro/Support</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/Support)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/Support)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -16269,7 +16269,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/TD</t>
+          <t>09_ai/AI_vai_tro/TD</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -16284,7 +16284,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/TD)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/TD)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -16307,7 +16307,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/UAV</t>
+          <t>09_ai/AI_vai_tro/UAV</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -16322,7 +16322,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/UAV)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/UAV)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -16345,7 +16345,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_vai_tro/VBIED</t>
+          <t>09_ai/AI_vai_tro/VBIED</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -16360,7 +16360,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/AI_vai_tro/VBIED)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/AI_vai_tro/VBIED)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -16383,7 +16383,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/air_superiority</t>
+          <t>09_ai/Chien_thuat/air_superiority</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -16398,7 +16398,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/air_superiority)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/air_superiority)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -16421,7 +16421,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/all_out</t>
+          <t>09_ai/Chien_thuat/all_out</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/all_out)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/all_out)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/ambush</t>
+          <t>09_ai/Chien_thuat/ambush</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/ambush)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/ambush)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -16497,7 +16497,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/attrition</t>
+          <t>09_ai/Chien_thuat/attrition</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -16512,7 +16512,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/attrition)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/attrition)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -16535,7 +16535,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/balanced</t>
+          <t>09_ai/Chien_thuat/balanced</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -16550,7 +16550,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/balanced)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/balanced)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -16573,7 +16573,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/base_defence</t>
+          <t>09_ai/Chien_thuat/base_defence</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -16588,7 +16588,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/base_defence)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/base_defence)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -16611,7 +16611,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/blitz</t>
+          <t>09_ai/Chien_thuat/blitz</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -16626,7 +16626,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/blitz)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/blitz)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -16649,7 +16649,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/bounding</t>
+          <t>09_ai/Chien_thuat/bounding</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -16664,7 +16664,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/bounding)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/bounding)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -16687,7 +16687,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/breakthrough</t>
+          <t>09_ai/Chien_thuat/breakthrough</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -16702,7 +16702,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/breakthrough)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/breakthrough)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -16725,7 +16725,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/decapitation</t>
+          <t>09_ai/Chien_thuat/decapitation</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -16740,7 +16740,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/decapitation)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/decapitation)</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -16763,7 +16763,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/depth</t>
+          <t>09_ai/Chien_thuat/depth</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -16778,7 +16778,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/depth)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/depth)</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -16801,7 +16801,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/dispersal</t>
+          <t>09_ai/Chien_thuat/dispersal</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -16816,7 +16816,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/dispersal)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/dispersal)</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -16839,7 +16839,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/encircle</t>
+          <t>09_ai/Chien_thuat/encircle</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -16854,7 +16854,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/encircle)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/encircle)</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -16877,7 +16877,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/firepower</t>
+          <t>09_ai/Chien_thuat/firepower</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -16892,7 +16892,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/firepower)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/firepower)</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -16915,7 +16915,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/hit_and_run</t>
+          <t>09_ai/Chien_thuat/hit_and_run</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -16930,7 +16930,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/hit_and_run)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/hit_and_run)</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/Chien_thuat/sead</t>
+          <t>09_ai/Chien_thuat/sead</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -16968,7 +16968,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (04_che_do_kinh_te_ai/Chien_thuat/sead)</t>
+          <t>Docs/ai/Machine_Brigade_AI_Research.xlsx (09_ai/Chien_thuat/sead)</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -30621,12 +30621,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu;04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu;09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat; Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu; 09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat; Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -30689,12 +30689,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -30723,12 +30723,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -30757,12 +30757,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat; Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat; Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -30859,12 +30859,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap;08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap;08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap; 08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap; 08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -30927,12 +30927,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -30995,12 +30995,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -31063,12 +31063,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap;04_che_do_kinh_te_ai/AI_tham_chieu;04_che_do_kinh_te_ai/AI_tham_so;04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap;09_ai/AI_tham_chieu;09_ai/AI_tham_so;09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap; 04_che_do_kinh_te_ai/AI_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_so; 04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap; 09_ai/AI_tham_chieu; 09_ai/AI_tham_so; 09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -31097,12 +31097,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap;04_che_do_kinh_te_ai/Che_do_tham_chieu;04_che_do_kinh_te_ai/AI_tham_chieu;04_che_do_kinh_te_ai/AI_tham_so;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap;04_che_do_kinh_te_ai/Che_do_tham_chieu;09_ai/AI_tham_chieu;09_ai/AI_tham_so;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap; 04_che_do_kinh_te_ai/Che_do_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_so; 08_tham_chieu/Tham_chieu_de_xuat; 1</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap; 04_che_do_kinh_te_ai/Che_do_tham_chieu; 09_ai/AI_tham_chieu; 09_ai/AI_tham_so; 08_tham_chieu/Tham_chieu_de_xuat; 1</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -31131,12 +31131,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -31199,12 +31199,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -31267,12 +31267,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -31335,12 +31335,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -31369,12 +31369,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/AI_tham_chieu;09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; 04_che_do_kinh_te_ai/Chien_thuat</t>
+          <t>09_ai/AI_tham_chieu; 09_ai/Chien_thuat</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -31403,12 +31403,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -31437,12 +31437,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -31471,12 +31471,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu;04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu;09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu; 09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -31573,12 +31573,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -31641,12 +31641,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -31777,12 +31777,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_tham_chieu;Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_tham_chieu; Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -31811,12 +31811,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>01_chien_dau/Phuong_tien_tham_chieu;03_can_cu/Can_cu_tham_chieu;04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>01_chien_dau/Phuong_tien_tham_chieu;03_can_cu/Can_cu_tham_chieu;09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>01_chien_dau/Phuong_tien_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>01_chien_dau/Phuong_tien_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -31845,12 +31845,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -31879,12 +31879,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>02_boss/Boss_tham_chieu;03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap;04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu;04_che_do_kinh_te_ai/AI_tham_chieu;04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>02_boss/Boss_tham_chieu;03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap;09_ai/AI_boss; 02_boss/Boss_tham_chieu;09_ai/AI_tham_chieu;09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>02_boss/Boss_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap; 04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_chieu; 04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>02_boss/Boss_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap; 09_ai/AI_boss; 02_boss/Boss_tham_chieu; 09_ai/AI_tham_chieu; 09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -31913,12 +31913,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -31947,12 +31947,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -31981,12 +31981,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -32015,12 +32015,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -32049,12 +32049,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_so</t>
+          <t>09_ai/AI_tham_so</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -32117,12 +32117,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat;Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat; Tham_chieu_decisions (ngoài gói)</t>
+          <t>09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat; Tham_chieu_decisions (ngoài gói)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -32185,12 +32185,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_tham_chieu</t>
+          <t>09_ai/AI_tham_chieu</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -32287,12 +32287,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap;04_che_do_kinh_te_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>03_can_cu/Can_cu_tham_chieu;03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap;09_ai/AI_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 04_che_do_kinh_te_ai/AI_thap; 04_che_do_kinh_te_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>03_can_cu/Can_cu_tham_chieu; 03_can_cu/Can_cu_tham_chieu; 09_ai/AI_thap; 09_ai/AI_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -32355,12 +32355,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu;08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>04_che_do_kinh_te_ai/AI_boss; 02_boss/Boss_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
+          <t>09_ai/AI_boss; 02_boss/Boss_tham_chieu; 08_tham_chieu/Tham_chieu_de_xuat</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>

</xml_diff>

<commit_message>
Export: rebuild the pack after the naval expansion, deck tabs and battleship triple turrets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/export/current/08_tham_chieu.xlsx
+++ b/Docs/export/current/08_tham_chieu.xlsx
@@ -19713,7 +19713,7 @@
       </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="n">
-        <v>735</v>
+        <v>754</v>
       </c>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
@@ -21633,7 +21633,7 @@
       </c>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="n">
-        <v>723</v>
+        <v>741</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -26261,7 +26261,7 @@
         </is>
       </c>
       <c r="K227" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L227" t="inlineStr">
         <is>
@@ -26549,7 +26549,7 @@
         </is>
       </c>
       <c r="K233" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L233" t="inlineStr">
         <is>
@@ -28897,7 +28897,7 @@
         </is>
       </c>
       <c r="K284" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L284" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Export: read Pack 2 tunables back into C# tables (inline SimTunables refs), conquest income regex; rebuild the pack
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/export/current/08_tham_chieu.xlsx
+++ b/Docs/export/current/08_tham_chieu.xlsx
@@ -19713,7 +19713,7 @@
       </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="n">
-        <v>754</v>
+        <v>785</v>
       </c>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
@@ -21633,7 +21633,7 @@
       </c>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="n">
-        <v>741</v>
+        <v>754</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -26213,7 +26213,7 @@
         </is>
       </c>
       <c r="K226" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -26789,7 +26789,7 @@
         </is>
       </c>
       <c r="K238" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -27485,7 +27485,7 @@
         </is>
       </c>
       <c r="K253" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -29221,7 +29221,7 @@
         </is>
       </c>
       <c r="K291" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -29545,7 +29545,7 @@
         </is>
       </c>
       <c r="K298" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L298" t="inlineStr">
         <is>

</xml_diff>